<commit_message>
add send email class
</commit_message>
<xml_diff>
--- a/src/main/resources/resultados_aprobaciones.xlsx
+++ b/src/main/resources/resultados_aprobaciones.xlsx
@@ -3,27 +3,25 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fredy\FdyAdla\fidu\fidugestor_aprobaciones\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fredy\FdyAdla\fidu\gestor_aprobaciones\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2362836D-EA4F-47AF-B37C-7C654B0D7184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14773A5F-1B8E-425E-9C20-3AAC121FD74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="resultados_09_03_26_20_09" sheetId="5" r:id="rId1"/>
     <sheet name="resultados_10_03_26_11_07" sheetId="8" r:id="rId2"/>
-    <sheet name="resultados_10_03_26_16_09" r:id="rId6" sheetId="9"/>
-    <sheet name="resultados_10_03_26_16_48" r:id="rId7" sheetId="10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="491">
   <si>
     <t>Referencia</t>
   </si>
@@ -1502,7 +1500,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1916,11 +1913,11 @@
   <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="38.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="29.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.28515625"/>
-    <col min="5" max="6" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" style="3" width="9.7109375"/>
+    <col min="1" max="1" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1947,22 +1944,22 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>288</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>287</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
         <v>286</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>285</v>
       </c>
       <c r="G2" s="3" t="s">
@@ -1970,22 +1967,22 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>284</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>283</v>
       </c>
-      <c r="C3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s" s="0">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>282</v>
       </c>
-      <c r="F3" t="s" s="0">
+      <c r="F3" t="s">
         <v>281</v>
       </c>
       <c r="G3" s="3" t="s">
@@ -1993,22 +1990,22 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>280</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>279</v>
       </c>
-      <c r="C4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s" s="0">
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>276</v>
       </c>
-      <c r="F4" t="s" s="0">
+      <c r="F4" t="s">
         <v>275</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -2016,22 +2013,22 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>278</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>277</v>
       </c>
-      <c r="C5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s" s="0">
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
         <v>276</v>
       </c>
-      <c r="F5" t="s" s="0">
+      <c r="F5" t="s">
         <v>275</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -2039,22 +2036,22 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>274</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>273</v>
       </c>
-      <c r="C6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E6" t="s" s="0">
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
         <v>272</v>
       </c>
-      <c r="F6" t="s" s="0">
+      <c r="F6" t="s">
         <v>271</v>
       </c>
       <c r="G6" s="3" t="s">
@@ -2062,22 +2059,22 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>270</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>269</v>
       </c>
-      <c r="C7" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s" s="0">
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
         <v>268</v>
       </c>
-      <c r="F7" t="s" s="0">
+      <c r="F7" t="s">
         <v>267</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -2085,22 +2082,22 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>266</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>265</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s" s="0">
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
         <v>264</v>
       </c>
-      <c r="F8" t="s" s="0">
+      <c r="F8" t="s">
         <v>263</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -2108,22 +2105,22 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>262</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>261</v>
       </c>
-      <c r="C9" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s" s="0">
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
         <v>252</v>
       </c>
-      <c r="F9" t="s" s="0">
+      <c r="F9" t="s">
         <v>251</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -2131,22 +2128,22 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>260</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>259</v>
       </c>
-      <c r="C10" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s" s="0">
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
         <v>252</v>
       </c>
-      <c r="F10" t="s" s="0">
+      <c r="F10" t="s">
         <v>251</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -2154,22 +2151,22 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>258</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>257</v>
       </c>
-      <c r="C11" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s" s="0">
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
         <v>256</v>
       </c>
-      <c r="F11" t="s" s="0">
+      <c r="F11" t="s">
         <v>255</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -2177,22 +2174,22 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>254</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>253</v>
       </c>
-      <c r="C12" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s" s="0">
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
         <v>252</v>
       </c>
-      <c r="F12" t="s" s="0">
+      <c r="F12" t="s">
         <v>251</v>
       </c>
       <c r="G12" s="3" t="s">
@@ -2200,22 +2197,22 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>7</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>8</v>
       </c>
-      <c r="C13" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s" s="0">
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
         <v>11</v>
       </c>
-      <c r="F13" t="s" s="0">
+      <c r="F13" t="s">
         <v>12</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -2223,22 +2220,22 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E14" t="s" s="0">
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
         <v>16</v>
       </c>
-      <c r="F14" t="s" s="0">
+      <c r="F14" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -2246,22 +2243,22 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>18</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>19</v>
       </c>
-      <c r="C15" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E15" t="s" s="0">
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
         <v>20</v>
       </c>
-      <c r="F15" t="s" s="0">
+      <c r="F15" t="s">
         <v>21</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -2269,22 +2266,22 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>22</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>23</v>
       </c>
-      <c r="C16" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E16" t="s" s="0">
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
         <v>24</v>
       </c>
-      <c r="F16" t="s" s="0">
+      <c r="F16" t="s">
         <v>25</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -2292,22 +2289,22 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
         <v>26</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>27</v>
       </c>
-      <c r="C17" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s" s="0">
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
         <v>28</v>
       </c>
-      <c r="F17" t="s" s="0">
+      <c r="F17" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -2315,22 +2312,22 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>30</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>31</v>
       </c>
-      <c r="C18" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E18" t="s" s="0">
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
         <v>32</v>
       </c>
-      <c r="F18" t="s" s="0">
+      <c r="F18" t="s">
         <v>33</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -2338,22 +2335,22 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>34</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E19" t="s" s="0">
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
         <v>36</v>
       </c>
-      <c r="F19" t="s" s="0">
+      <c r="F19" t="s">
         <v>37</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -2361,22 +2358,22 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>39</v>
       </c>
-      <c r="C20" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E20" t="s" s="0">
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s">
         <v>40</v>
       </c>
-      <c r="F20" t="s" s="0">
+      <c r="F20" t="s">
         <v>41</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -2384,22 +2381,22 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>42</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>43</v>
       </c>
-      <c r="C21" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E21" t="s" s="0">
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
         <v>44</v>
       </c>
-      <c r="F21" t="s" s="0">
+      <c r="F21" t="s">
         <v>45</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -2407,22 +2404,22 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>46</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>47</v>
       </c>
-      <c r="C22" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E22" t="s" s="0">
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
         <v>44</v>
       </c>
-      <c r="F22" t="s" s="0">
+      <c r="F22" t="s">
         <v>45</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -2430,22 +2427,22 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>48</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>49</v>
       </c>
-      <c r="C23" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E23" t="s" s="0">
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
         <v>50</v>
       </c>
-      <c r="F23" t="s" s="0">
+      <c r="F23" t="s">
         <v>51</v>
       </c>
       <c r="G23" s="3" t="s">
@@ -2453,22 +2450,22 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>52</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>53</v>
       </c>
-      <c r="C24" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E24" t="s" s="0">
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
         <v>54</v>
       </c>
-      <c r="F24" t="s" s="0">
+      <c r="F24" t="s">
         <v>55</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -2476,22 +2473,22 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s" s="0">
+      <c r="A25" t="s">
         <v>56</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="C25" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E25" t="s" s="0">
+      <c r="C25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
         <v>58</v>
       </c>
-      <c r="F25" t="s" s="0">
+      <c r="F25" t="s">
         <v>59</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -2499,22 +2496,22 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s" s="0">
+      <c r="A26" t="s">
         <v>60</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>61</v>
       </c>
-      <c r="C26" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D26" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E26" t="s" s="0">
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s">
         <v>62</v>
       </c>
-      <c r="F26" t="s" s="0">
+      <c r="F26" t="s">
         <v>63</v>
       </c>
       <c r="G26" s="3" t="s">
@@ -2522,22 +2519,22 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s" s="0">
+      <c r="A27" t="s">
         <v>64</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>65</v>
       </c>
-      <c r="C27" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E27" t="s" s="0">
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
         <v>62</v>
       </c>
-      <c r="F27" t="s" s="0">
+      <c r="F27" t="s">
         <v>63</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -2545,22 +2542,22 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s" s="0">
+      <c r="A28" t="s">
         <v>66</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E28" t="s" s="0">
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s">
         <v>68</v>
       </c>
-      <c r="F28" t="s" s="0">
+      <c r="F28" t="s">
         <v>69</v>
       </c>
       <c r="G28" s="3" t="s">
@@ -2568,22 +2565,22 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s" s="0">
+      <c r="A29" t="s">
         <v>70</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>71</v>
       </c>
-      <c r="C29" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D29" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E29" t="s" s="0">
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
         <v>68</v>
       </c>
-      <c r="F29" t="s" s="0">
+      <c r="F29" t="s">
         <v>69</v>
       </c>
       <c r="G29" s="3" t="s">
@@ -2591,22 +2588,22 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s" s="0">
+      <c r="A30" t="s">
         <v>72</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>73</v>
       </c>
-      <c r="C30" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D30" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E30" t="s" s="0">
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s">
         <v>74</v>
       </c>
-      <c r="F30" t="s" s="0">
+      <c r="F30" t="s">
         <v>75</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -2614,22 +2611,22 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" t="s" s="0">
+      <c r="A31" t="s">
         <v>76</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>77</v>
       </c>
-      <c r="C31" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D31" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E31" t="s" s="0">
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
         <v>78</v>
       </c>
-      <c r="F31" t="s" s="0">
+      <c r="F31" t="s">
         <v>79</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -2637,22 +2634,22 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" t="s" s="0">
+      <c r="A32" t="s">
         <v>80</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>81</v>
       </c>
-      <c r="C32" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E32" t="s" s="0">
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" t="s">
         <v>78</v>
       </c>
-      <c r="F32" t="s" s="0">
+      <c r="F32" t="s">
         <v>79</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -2660,22 +2657,22 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s" s="0">
+      <c r="A33" t="s">
         <v>82</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>83</v>
       </c>
-      <c r="C33" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E33" t="s" s="0">
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s">
         <v>84</v>
       </c>
-      <c r="F33" t="s" s="0">
+      <c r="F33" t="s">
         <v>85</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -2683,22 +2680,22 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s" s="0">
+      <c r="A34" t="s">
         <v>86</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>87</v>
       </c>
-      <c r="C34" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D34" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E34" t="s" s="0">
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" t="s">
         <v>88</v>
       </c>
-      <c r="F34" t="s" s="0">
+      <c r="F34" t="s">
         <v>89</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -2706,22 +2703,22 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s" s="0">
+      <c r="A35" t="s">
         <v>90</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>91</v>
       </c>
-      <c r="C35" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D35" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E35" t="s" s="0">
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
         <v>92</v>
       </c>
-      <c r="F35" t="s" s="0">
+      <c r="F35" t="s">
         <v>93</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -2729,22 +2726,22 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s" s="0">
+      <c r="A36" t="s">
         <v>94</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>95</v>
       </c>
-      <c r="C36" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D36" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E36" t="s" s="0">
+      <c r="C36" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
         <v>96</v>
       </c>
-      <c r="F36" t="s" s="0">
+      <c r="F36" t="s">
         <v>97</v>
       </c>
       <c r="G36" s="3" t="s">
@@ -2752,22 +2749,22 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s" s="0">
+      <c r="A37" t="s">
         <v>98</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>99</v>
       </c>
-      <c r="C37" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D37" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E37" t="s" s="0">
+      <c r="C37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" t="s">
         <v>100</v>
       </c>
-      <c r="F37" t="s" s="0">
+      <c r="F37" t="s">
         <v>101</v>
       </c>
       <c r="G37" s="3" t="s">
@@ -2775,22 +2772,22 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" t="s" s="0">
+      <c r="A38" t="s">
         <v>102</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>103</v>
       </c>
-      <c r="C38" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D38" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E38" t="s" s="0">
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" t="s">
         <v>104</v>
       </c>
-      <c r="F38" t="s" s="0">
+      <c r="F38" t="s">
         <v>105</v>
       </c>
       <c r="G38" s="3" t="s">
@@ -2798,22 +2795,22 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" t="s" s="0">
+      <c r="A39" t="s">
         <v>106</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>107</v>
       </c>
-      <c r="C39" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D39" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E39" t="s" s="0">
+      <c r="C39" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
         <v>108</v>
       </c>
-      <c r="F39" t="s" s="0">
+      <c r="F39" t="s">
         <v>109</v>
       </c>
       <c r="G39" s="3" t="s">
@@ -2821,22 +2818,22 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" t="s" s="0">
+      <c r="A40" t="s">
         <v>110</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>111</v>
       </c>
-      <c r="C40" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D40" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E40" t="s" s="0">
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" t="s">
         <v>112</v>
       </c>
-      <c r="F40" t="s" s="0">
+      <c r="F40" t="s">
         <v>113</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -2844,22 +2841,22 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" t="s" s="0">
+      <c r="A41" t="s">
         <v>114</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>115</v>
       </c>
-      <c r="C41" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D41" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E41" t="s" s="0">
+      <c r="C41" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s">
         <v>116</v>
       </c>
-      <c r="F41" t="s" s="0">
+      <c r="F41" t="s">
         <v>117</v>
       </c>
       <c r="G41" s="3" t="s">
@@ -2867,22 +2864,22 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s" s="0">
+      <c r="A42" t="s">
         <v>118</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>119</v>
       </c>
-      <c r="C42" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E42" t="s" s="0">
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" t="s">
         <v>116</v>
       </c>
-      <c r="F42" t="s" s="0">
+      <c r="F42" t="s">
         <v>117</v>
       </c>
       <c r="G42" s="3" t="s">
@@ -2890,22 +2887,22 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s" s="0">
+      <c r="A43" t="s">
         <v>120</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>121</v>
       </c>
-      <c r="C43" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D43" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E43" t="s" s="0">
+      <c r="C43" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s">
         <v>122</v>
       </c>
-      <c r="F43" t="s" s="0">
+      <c r="F43" t="s">
         <v>123</v>
       </c>
       <c r="G43" s="3" t="s">
@@ -2913,22 +2910,22 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" t="s" s="0">
+      <c r="A44" t="s">
         <v>124</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>125</v>
       </c>
-      <c r="C44" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D44" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E44" t="s" s="0">
+      <c r="C44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" t="s">
         <v>126</v>
       </c>
-      <c r="F44" t="s" s="0">
+      <c r="F44" t="s">
         <v>127</v>
       </c>
       <c r="G44" s="3" t="s">
@@ -2936,22 +2933,22 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="s" s="0">
+      <c r="A45" t="s">
         <v>128</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>129</v>
       </c>
-      <c r="C45" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D45" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E45" t="s" s="0">
+      <c r="C45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" t="s">
         <v>130</v>
       </c>
-      <c r="F45" t="s" s="0">
+      <c r="F45" t="s">
         <v>131</v>
       </c>
       <c r="G45" s="3" t="s">
@@ -2959,22 +2956,22 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="s" s="0">
+      <c r="A46" t="s">
         <v>132</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>133</v>
       </c>
-      <c r="C46" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D46" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E46" t="s" s="0">
+      <c r="C46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
         <v>130</v>
       </c>
-      <c r="F46" t="s" s="0">
+      <c r="F46" t="s">
         <v>131</v>
       </c>
       <c r="G46" s="3" t="s">
@@ -2982,22 +2979,22 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" t="s" s="0">
+      <c r="A47" t="s">
         <v>134</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>135</v>
       </c>
-      <c r="C47" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D47" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E47" t="s" s="0">
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s">
         <v>136</v>
       </c>
-      <c r="F47" t="s" s="0">
+      <c r="F47" t="s">
         <v>137</v>
       </c>
       <c r="G47" s="3" t="s">
@@ -3005,22 +3002,22 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" t="s" s="0">
+      <c r="A48" t="s">
         <v>138</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>139</v>
       </c>
-      <c r="C48" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E48" t="s" s="0">
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" t="s">
         <v>140</v>
       </c>
-      <c r="F48" t="s" s="0">
+      <c r="F48" t="s">
         <v>141</v>
       </c>
       <c r="G48" s="3" t="s">
@@ -3028,22 +3025,22 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" t="s" s="0">
+      <c r="A49" t="s">
         <v>142</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>143</v>
       </c>
-      <c r="C49" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D49" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E49" t="s" s="0">
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s">
         <v>144</v>
       </c>
-      <c r="F49" t="s" s="0">
+      <c r="F49" t="s">
         <v>145</v>
       </c>
       <c r="G49" s="3" t="s">
@@ -3051,22 +3048,22 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" t="s" s="0">
+      <c r="A50" t="s">
         <v>146</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>147</v>
       </c>
-      <c r="C50" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D50" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E50" t="s" s="0">
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s">
         <v>148</v>
       </c>
-      <c r="F50" t="s" s="0">
+      <c r="F50" t="s">
         <v>149</v>
       </c>
       <c r="G50" s="3" t="s">
@@ -3074,22 +3071,22 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" t="s" s="0">
+      <c r="A51" t="s">
         <v>150</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>151</v>
       </c>
-      <c r="C51" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D51" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E51" t="s" s="0">
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s">
         <v>148</v>
       </c>
-      <c r="F51" t="s" s="0">
+      <c r="F51" t="s">
         <v>149</v>
       </c>
       <c r="G51" s="3" t="s">
@@ -3097,22 +3094,22 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s" s="0">
+      <c r="A52" t="s">
         <v>152</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>153</v>
       </c>
-      <c r="C52" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D52" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E52" t="s" s="0">
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
         <v>154</v>
       </c>
-      <c r="F52" t="s" s="0">
+      <c r="F52" t="s">
         <v>155</v>
       </c>
       <c r="G52" s="3" t="s">
@@ -3120,22 +3117,22 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s" s="0">
+      <c r="A53" t="s">
         <v>156</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>157</v>
       </c>
-      <c r="C53" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D53" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E53" t="s" s="0">
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
         <v>158</v>
       </c>
-      <c r="F53" t="s" s="0">
+      <c r="F53" t="s">
         <v>159</v>
       </c>
       <c r="G53" s="3" t="s">
@@ -3143,22 +3140,22 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" t="s" s="0">
+      <c r="A54" t="s">
         <v>160</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>161</v>
       </c>
-      <c r="C54" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D54" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E54" t="s" s="0">
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" t="s">
         <v>162</v>
       </c>
-      <c r="F54" t="s" s="0">
+      <c r="F54" t="s">
         <v>163</v>
       </c>
       <c r="G54" s="3" t="s">
@@ -3166,22 +3163,22 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s" s="0">
+      <c r="A55" t="s">
         <v>164</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>165</v>
       </c>
-      <c r="C55" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D55" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E55" t="s" s="0">
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
         <v>166</v>
       </c>
-      <c r="F55" t="s" s="0">
+      <c r="F55" t="s">
         <v>167</v>
       </c>
       <c r="G55" s="3" t="s">
@@ -3189,22 +3186,22 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s" s="0">
+      <c r="A56" t="s">
         <v>168</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>169</v>
       </c>
-      <c r="C56" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D56" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E56" t="s" s="0">
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" t="s">
         <v>170</v>
       </c>
-      <c r="F56" t="s" s="0">
+      <c r="F56" t="s">
         <v>171</v>
       </c>
       <c r="G56" s="3" t="s">
@@ -3212,22 +3209,22 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s" s="0">
+      <c r="A57" t="s">
         <v>172</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>173</v>
       </c>
-      <c r="C57" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D57" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E57" t="s" s="0">
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
         <v>174</v>
       </c>
-      <c r="F57" t="s" s="0">
+      <c r="F57" t="s">
         <v>175</v>
       </c>
       <c r="G57" s="3" t="s">
@@ -3235,22 +3232,22 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s" s="0">
+      <c r="A58" t="s">
         <v>176</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B58" t="s">
         <v>177</v>
       </c>
-      <c r="C58" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D58" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E58" t="s" s="0">
+      <c r="C58" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s">
+        <v>10</v>
+      </c>
+      <c r="E58" t="s">
         <v>178</v>
       </c>
-      <c r="F58" t="s" s="0">
+      <c r="F58" t="s">
         <v>179</v>
       </c>
       <c r="G58" s="3" t="s">
@@ -3258,22 +3255,22 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" t="s" s="0">
+      <c r="A59" t="s">
         <v>180</v>
       </c>
-      <c r="B59" t="s" s="0">
+      <c r="B59" t="s">
         <v>181</v>
       </c>
-      <c r="C59" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D59" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E59" t="s" s="0">
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s">
+        <v>10</v>
+      </c>
+      <c r="E59" t="s">
         <v>182</v>
       </c>
-      <c r="F59" t="s" s="0">
+      <c r="F59" t="s">
         <v>183</v>
       </c>
       <c r="G59" s="3" t="s">
@@ -3281,22 +3278,22 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" t="s" s="0">
+      <c r="A60" t="s">
         <v>184</v>
       </c>
-      <c r="B60" t="s" s="0">
+      <c r="B60" t="s">
         <v>185</v>
       </c>
-      <c r="C60" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D60" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E60" t="s" s="0">
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>10</v>
+      </c>
+      <c r="E60" t="s">
         <v>186</v>
       </c>
-      <c r="F60" t="s" s="0">
+      <c r="F60" t="s">
         <v>187</v>
       </c>
       <c r="G60" s="3" t="s">
@@ -3304,22 +3301,22 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" t="s" s="0">
+      <c r="A61" t="s">
         <v>188</v>
       </c>
-      <c r="B61" t="s" s="0">
+      <c r="B61" t="s">
         <v>189</v>
       </c>
-      <c r="C61" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D61" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E61" t="s" s="0">
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" t="s">
         <v>190</v>
       </c>
-      <c r="F61" t="s" s="0">
+      <c r="F61" t="s">
         <v>191</v>
       </c>
       <c r="G61" s="3" t="s">
@@ -3327,22 +3324,22 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" t="s" s="0">
+      <c r="A62" t="s">
         <v>192</v>
       </c>
-      <c r="B62" t="s" s="0">
+      <c r="B62" t="s">
         <v>193</v>
       </c>
-      <c r="C62" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D62" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E62" t="s" s="0">
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s">
+        <v>10</v>
+      </c>
+      <c r="E62" t="s">
         <v>194</v>
       </c>
-      <c r="F62" t="s" s="0">
+      <c r="F62" t="s">
         <v>195</v>
       </c>
       <c r="G62" s="3" t="s">
@@ -3350,22 +3347,22 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s" s="0">
+      <c r="A63" t="s">
         <v>196</v>
       </c>
-      <c r="B63" t="s" s="0">
+      <c r="B63" t="s">
         <v>197</v>
       </c>
-      <c r="C63" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D63" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E63" t="s" s="0">
+      <c r="C63" t="s">
+        <v>9</v>
+      </c>
+      <c r="D63" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" t="s">
         <v>198</v>
       </c>
-      <c r="F63" t="s" s="0">
+      <c r="F63" t="s">
         <v>199</v>
       </c>
       <c r="G63" s="3" t="s">
@@ -3373,22 +3370,22 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" t="s" s="0">
+      <c r="A64" t="s">
         <v>200</v>
       </c>
-      <c r="B64" t="s" s="0">
+      <c r="B64" t="s">
         <v>201</v>
       </c>
-      <c r="C64" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D64" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E64" t="s" s="0">
+      <c r="C64" t="s">
+        <v>9</v>
+      </c>
+      <c r="D64" t="s">
+        <v>10</v>
+      </c>
+      <c r="E64" t="s">
         <v>202</v>
       </c>
-      <c r="F64" t="s" s="0">
+      <c r="F64" t="s">
         <v>203</v>
       </c>
       <c r="G64" s="3" t="s">
@@ -3396,22 +3393,22 @@
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" t="s" s="0">
+      <c r="A65" t="s">
         <v>204</v>
       </c>
-      <c r="B65" t="s" s="0">
+      <c r="B65" t="s">
         <v>205</v>
       </c>
-      <c r="C65" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D65" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E65" t="s" s="0">
+      <c r="C65" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" t="s">
+        <v>10</v>
+      </c>
+      <c r="E65" t="s">
         <v>202</v>
       </c>
-      <c r="F65" t="s" s="0">
+      <c r="F65" t="s">
         <v>203</v>
       </c>
       <c r="G65" s="3" t="s">
@@ -3419,22 +3416,22 @@
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="s" s="0">
+      <c r="A66" t="s">
         <v>206</v>
       </c>
-      <c r="B66" t="s" s="0">
+      <c r="B66" t="s">
         <v>207</v>
       </c>
-      <c r="C66" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D66" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E66" t="s" s="0">
+      <c r="C66" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" t="s">
+        <v>10</v>
+      </c>
+      <c r="E66" t="s">
         <v>208</v>
       </c>
-      <c r="F66" t="s" s="0">
+      <c r="F66" t="s">
         <v>209</v>
       </c>
       <c r="G66" s="3" t="s">
@@ -3442,22 +3439,22 @@
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="s" s="0">
+      <c r="A67" t="s">
         <v>210</v>
       </c>
-      <c r="B67" t="s" s="0">
+      <c r="B67" t="s">
         <v>211</v>
       </c>
-      <c r="C67" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D67" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E67" t="s" s="0">
+      <c r="C67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D67" t="s">
+        <v>10</v>
+      </c>
+      <c r="E67" t="s">
         <v>212</v>
       </c>
-      <c r="F67" t="s" s="0">
+      <c r="F67" t="s">
         <v>213</v>
       </c>
       <c r="G67" s="3" t="s">
@@ -3465,22 +3462,22 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s" s="0">
+      <c r="A68" t="s">
         <v>214</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B68" t="s">
         <v>215</v>
       </c>
-      <c r="C68" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D68" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E68" t="s" s="0">
+      <c r="C68" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" t="s">
+        <v>10</v>
+      </c>
+      <c r="E68" t="s">
         <v>216</v>
       </c>
-      <c r="F68" t="s" s="0">
+      <c r="F68" t="s">
         <v>217</v>
       </c>
       <c r="G68" s="3" t="s">
@@ -3488,22 +3485,22 @@
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="s" s="0">
+      <c r="A69" t="s">
         <v>218</v>
       </c>
-      <c r="B69" t="s" s="0">
+      <c r="B69" t="s">
         <v>219</v>
       </c>
-      <c r="C69" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D69" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E69" t="s" s="0">
+      <c r="C69" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" t="s">
+        <v>10</v>
+      </c>
+      <c r="E69" t="s">
         <v>148</v>
       </c>
-      <c r="F69" t="s" s="0">
+      <c r="F69" t="s">
         <v>149</v>
       </c>
       <c r="G69" s="3" t="s">
@@ -3511,22 +3508,22 @@
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" t="s" s="0">
+      <c r="A70" t="s">
         <v>220</v>
       </c>
-      <c r="B70" t="s" s="0">
+      <c r="B70" t="s">
         <v>221</v>
       </c>
-      <c r="C70" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D70" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E70" t="s" s="0">
+      <c r="C70" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" t="s">
+        <v>10</v>
+      </c>
+      <c r="E70" t="s">
         <v>222</v>
       </c>
-      <c r="F70" t="s" s="0">
+      <c r="F70" t="s">
         <v>195</v>
       </c>
       <c r="G70" s="3" t="s">
@@ -3534,22 +3531,22 @@
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" t="s" s="0">
+      <c r="A71" t="s">
         <v>223</v>
       </c>
-      <c r="B71" t="s" s="0">
+      <c r="B71" t="s">
         <v>224</v>
       </c>
-      <c r="C71" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D71" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E71" t="s" s="0">
+      <c r="C71" t="s">
+        <v>9</v>
+      </c>
+      <c r="D71" t="s">
+        <v>10</v>
+      </c>
+      <c r="E71" t="s">
         <v>225</v>
       </c>
-      <c r="F71" t="s" s="0">
+      <c r="F71" t="s">
         <v>195</v>
       </c>
       <c r="G71" s="3" t="s">
@@ -3557,22 +3554,22 @@
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" t="s" s="0">
+      <c r="A72" t="s">
         <v>226</v>
       </c>
-      <c r="B72" t="s" s="0">
+      <c r="B72" t="s">
         <v>227</v>
       </c>
-      <c r="C72" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D72" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E72" t="s" s="0">
+      <c r="C72" t="s">
+        <v>9</v>
+      </c>
+      <c r="D72" t="s">
+        <v>10</v>
+      </c>
+      <c r="E72" t="s">
         <v>228</v>
       </c>
-      <c r="F72" t="s" s="0">
+      <c r="F72" t="s">
         <v>195</v>
       </c>
       <c r="G72" s="3" t="s">
@@ -3580,22 +3577,22 @@
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" t="s" s="0">
+      <c r="A73" t="s">
         <v>229</v>
       </c>
-      <c r="B73" t="s" s="0">
+      <c r="B73" t="s">
         <v>230</v>
       </c>
-      <c r="C73" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D73" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E73" t="s" s="0">
+      <c r="C73" t="s">
+        <v>9</v>
+      </c>
+      <c r="D73" t="s">
+        <v>10</v>
+      </c>
+      <c r="E73" t="s">
         <v>231</v>
       </c>
-      <c r="F73" t="s" s="0">
+      <c r="F73" t="s">
         <v>195</v>
       </c>
       <c r="G73" s="3" t="s">
@@ -3603,22 +3600,22 @@
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" t="s" s="0">
+      <c r="A74" t="s">
         <v>232</v>
       </c>
-      <c r="B74" t="s" s="0">
+      <c r="B74" t="s">
         <v>233</v>
       </c>
-      <c r="C74" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D74" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E74" t="s" s="0">
+      <c r="C74" t="s">
+        <v>9</v>
+      </c>
+      <c r="D74" t="s">
+        <v>10</v>
+      </c>
+      <c r="E74" t="s">
         <v>234</v>
       </c>
-      <c r="F74" t="s" s="0">
+      <c r="F74" t="s">
         <v>195</v>
       </c>
       <c r="G74" s="3" t="s">
@@ -3626,22 +3623,22 @@
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" t="s" s="0">
+      <c r="A75" t="s">
         <v>235</v>
       </c>
-      <c r="B75" t="s" s="0">
+      <c r="B75" t="s">
         <v>236</v>
       </c>
-      <c r="C75" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D75" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E75" t="s" s="0">
+      <c r="C75" t="s">
+        <v>9</v>
+      </c>
+      <c r="D75" t="s">
+        <v>10</v>
+      </c>
+      <c r="E75" t="s">
         <v>237</v>
       </c>
-      <c r="F75" t="s" s="0">
+      <c r="F75" t="s">
         <v>195</v>
       </c>
       <c r="G75" s="3" t="s">
@@ -3649,22 +3646,22 @@
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" t="s" s="0">
+      <c r="A76" t="s">
         <v>238</v>
       </c>
-      <c r="B76" t="s" s="0">
+      <c r="B76" t="s">
         <v>239</v>
       </c>
-      <c r="C76" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D76" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E76" t="s" s="0">
+      <c r="C76" t="s">
+        <v>9</v>
+      </c>
+      <c r="D76" t="s">
+        <v>10</v>
+      </c>
+      <c r="E76" t="s">
         <v>240</v>
       </c>
-      <c r="F76" t="s" s="0">
+      <c r="F76" t="s">
         <v>195</v>
       </c>
       <c r="G76" s="3" t="s">
@@ -3672,22 +3669,22 @@
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" t="s" s="0">
+      <c r="A77" t="s">
         <v>241</v>
       </c>
-      <c r="B77" t="s" s="0">
+      <c r="B77" t="s">
         <v>242</v>
       </c>
-      <c r="C77" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D77" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E77" t="s" s="0">
+      <c r="C77" t="s">
+        <v>9</v>
+      </c>
+      <c r="D77" t="s">
+        <v>10</v>
+      </c>
+      <c r="E77" t="s">
         <v>243</v>
       </c>
-      <c r="F77" t="s" s="0">
+      <c r="F77" t="s">
         <v>195</v>
       </c>
       <c r="G77" s="3" t="s">
@@ -3695,22 +3692,22 @@
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" t="s" s="0">
+      <c r="A78" t="s">
         <v>244</v>
       </c>
-      <c r="B78" t="s" s="0">
+      <c r="B78" t="s">
         <v>245</v>
       </c>
-      <c r="C78" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D78" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E78" t="s" s="0">
+      <c r="C78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D78" t="s">
+        <v>10</v>
+      </c>
+      <c r="E78" t="s">
         <v>246</v>
       </c>
-      <c r="F78" t="s" s="0">
+      <c r="F78" t="s">
         <v>195</v>
       </c>
       <c r="G78" s="3" t="s">
@@ -3718,22 +3715,22 @@
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" t="s" s="0">
+      <c r="A79" t="s">
         <v>247</v>
       </c>
-      <c r="B79" t="s" s="0">
+      <c r="B79" t="s">
         <v>248</v>
       </c>
-      <c r="C79" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D79" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E79" t="s" s="0">
+      <c r="C79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D79" t="s">
+        <v>10</v>
+      </c>
+      <c r="E79" t="s">
         <v>249</v>
       </c>
-      <c r="F79" t="s" s="0">
+      <c r="F79" t="s">
         <v>250</v>
       </c>
       <c r="G79" s="3" t="s">
@@ -3742,39 +3739,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s" s="0">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -3783,11 +3747,11 @@
   <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="38.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="29.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.42578125"/>
-    <col min="5" max="6" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="1" max="1" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -3814,22 +3778,22 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>292</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>293</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
         <v>290</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>291</v>
       </c>
       <c r="G2" s="3" t="s">
@@ -3837,22 +3801,22 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>294</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>295</v>
       </c>
-      <c r="C3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s" s="0">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>296</v>
       </c>
-      <c r="F3" t="s" s="0">
+      <c r="F3" t="s">
         <v>297</v>
       </c>
       <c r="G3" s="3" t="s">
@@ -3860,22 +3824,22 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>298</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>299</v>
       </c>
-      <c r="C4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s" s="0">
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>296</v>
       </c>
-      <c r="F4" t="s" s="0">
+      <c r="F4" t="s">
         <v>297</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -3883,22 +3847,22 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>300</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>301</v>
       </c>
-      <c r="C5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s" s="0">
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
         <v>302</v>
       </c>
-      <c r="F5" t="s" s="0">
+      <c r="F5" t="s">
         <v>303</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -3906,22 +3870,22 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>304</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>305</v>
       </c>
-      <c r="C6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E6" t="s" s="0">
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
         <v>306</v>
       </c>
-      <c r="F6" t="s" s="0">
+      <c r="F6" t="s">
         <v>307</v>
       </c>
       <c r="G6" s="3" t="s">
@@ -3929,22 +3893,22 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>308</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>309</v>
       </c>
-      <c r="C7" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s" s="0">
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
         <v>306</v>
       </c>
-      <c r="F7" t="s" s="0">
+      <c r="F7" t="s">
         <v>307</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -3952,22 +3916,22 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>310</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>311</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s" s="0">
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
         <v>306</v>
       </c>
-      <c r="F8" t="s" s="0">
+      <c r="F8" t="s">
         <v>307</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -3975,22 +3939,22 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>312</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>313</v>
       </c>
-      <c r="C9" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s" s="0">
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
         <v>314</v>
       </c>
-      <c r="F9" t="s" s="0">
+      <c r="F9" t="s">
         <v>315</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -3998,22 +3962,22 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>316</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s">
         <v>317</v>
       </c>
-      <c r="C10" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s" s="0">
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
         <v>318</v>
       </c>
-      <c r="F10" t="s" s="0">
+      <c r="F10" t="s">
         <v>195</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -4021,22 +3985,22 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>319</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s">
         <v>320</v>
       </c>
-      <c r="C11" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s" s="0">
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
         <v>321</v>
       </c>
-      <c r="F11" t="s" s="0">
+      <c r="F11" t="s">
         <v>195</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -4044,22 +4008,22 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>322</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s">
         <v>323</v>
       </c>
-      <c r="C12" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D12" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s" s="0">
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
         <v>324</v>
       </c>
-      <c r="F12" t="s" s="0">
+      <c r="F12" t="s">
         <v>325</v>
       </c>
       <c r="G12" s="3" t="s">
@@ -4067,22 +4031,22 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>289</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="B13" t="s">
         <v>326</v>
       </c>
-      <c r="C13" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D13" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s" s="0">
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
         <v>327</v>
       </c>
-      <c r="F13" t="s" s="0">
+      <c r="F13" t="s">
         <v>328</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -4090,22 +4054,22 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>329</v>
       </c>
-      <c r="B14" t="s" s="0">
+      <c r="B14" t="s">
         <v>330</v>
       </c>
-      <c r="C14" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E14" t="s" s="0">
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
         <v>331</v>
       </c>
-      <c r="F14" t="s" s="0">
+      <c r="F14" t="s">
         <v>332</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -4113,22 +4077,22 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>333</v>
       </c>
-      <c r="B15" t="s" s="0">
+      <c r="B15" t="s">
         <v>334</v>
       </c>
-      <c r="C15" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E15" t="s" s="0">
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
         <v>335</v>
       </c>
-      <c r="F15" t="s" s="0">
+      <c r="F15" t="s">
         <v>336</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -4136,22 +4100,22 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>337</v>
       </c>
-      <c r="B16" t="s" s="0">
+      <c r="B16" t="s">
         <v>338</v>
       </c>
-      <c r="C16" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E16" t="s" s="0">
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
         <v>339</v>
       </c>
-      <c r="F16" t="s" s="0">
+      <c r="F16" t="s">
         <v>340</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -4159,22 +4123,22 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s" s="0">
+      <c r="A17" t="s">
         <v>341</v>
       </c>
-      <c r="B17" t="s" s="0">
+      <c r="B17" t="s">
         <v>342</v>
       </c>
-      <c r="C17" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s" s="0">
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
         <v>343</v>
       </c>
-      <c r="F17" t="s" s="0">
+      <c r="F17" t="s">
         <v>344</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -4182,22 +4146,22 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s" s="0">
+      <c r="A18" t="s">
         <v>345</v>
       </c>
-      <c r="B18" t="s" s="0">
+      <c r="B18" t="s">
         <v>346</v>
       </c>
-      <c r="C18" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E18" t="s" s="0">
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
         <v>347</v>
       </c>
-      <c r="F18" t="s" s="0">
+      <c r="F18" t="s">
         <v>348</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -4205,22 +4169,22 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s" s="0">
+      <c r="A19" t="s">
         <v>349</v>
       </c>
-      <c r="B19" t="s" s="0">
+      <c r="B19" t="s">
         <v>350</v>
       </c>
-      <c r="C19" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D19" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E19" t="s" s="0">
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
         <v>351</v>
       </c>
-      <c r="F19" t="s" s="0">
+      <c r="F19" t="s">
         <v>352</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -4228,22 +4192,22 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s" s="0">
+      <c r="A20" t="s">
         <v>353</v>
       </c>
-      <c r="B20" t="s" s="0">
+      <c r="B20" t="s">
         <v>354</v>
       </c>
-      <c r="C20" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E20" t="s" s="0">
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s">
         <v>355</v>
       </c>
-      <c r="F20" t="s" s="0">
+      <c r="F20" t="s">
         <v>356</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -4251,22 +4215,22 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s" s="0">
+      <c r="A21" t="s">
         <v>357</v>
       </c>
-      <c r="B21" t="s" s="0">
+      <c r="B21" t="s">
         <v>358</v>
       </c>
-      <c r="C21" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E21" t="s" s="0">
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
         <v>355</v>
       </c>
-      <c r="F21" t="s" s="0">
+      <c r="F21" t="s">
         <v>356</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -4274,22 +4238,22 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s" s="0">
+      <c r="A22" t="s">
         <v>359</v>
       </c>
-      <c r="B22" t="s" s="0">
+      <c r="B22" t="s">
         <v>360</v>
       </c>
-      <c r="C22" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D22" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E22" t="s" s="0">
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
         <v>361</v>
       </c>
-      <c r="F22" t="s" s="0">
+      <c r="F22" t="s">
         <v>362</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -4297,22 +4261,22 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s" s="0">
+      <c r="A23" t="s">
         <v>363</v>
       </c>
-      <c r="B23" t="s" s="0">
+      <c r="B23" t="s">
         <v>364</v>
       </c>
-      <c r="C23" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D23" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E23" t="s" s="0">
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
         <v>365</v>
       </c>
-      <c r="F23" t="s" s="0">
+      <c r="F23" t="s">
         <v>366</v>
       </c>
       <c r="G23" s="3" t="s">
@@ -4320,22 +4284,22 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s" s="0">
+      <c r="A24" t="s">
         <v>367</v>
       </c>
-      <c r="B24" t="s" s="0">
+      <c r="B24" t="s">
         <v>368</v>
       </c>
-      <c r="C24" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D24" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E24" t="s" s="0">
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
         <v>369</v>
       </c>
-      <c r="F24" t="s" s="0">
+      <c r="F24" t="s">
         <v>370</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -4343,22 +4307,22 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s" s="0">
+      <c r="A25" t="s">
         <v>371</v>
       </c>
-      <c r="B25" t="s" s="0">
+      <c r="B25" t="s">
         <v>372</v>
       </c>
-      <c r="C25" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D25" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E25" t="s" s="0">
+      <c r="C25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
         <v>373</v>
       </c>
-      <c r="F25" t="s" s="0">
+      <c r="F25" t="s">
         <v>374</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -4366,22 +4330,22 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s" s="0">
+      <c r="A26" t="s">
         <v>375</v>
       </c>
-      <c r="B26" t="s" s="0">
+      <c r="B26" t="s">
         <v>376</v>
       </c>
-      <c r="C26" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D26" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E26" t="s" s="0">
+      <c r="C26" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s">
         <v>377</v>
       </c>
-      <c r="F26" t="s" s="0">
+      <c r="F26" t="s">
         <v>378</v>
       </c>
       <c r="G26" s="3" t="s">
@@ -4389,22 +4353,22 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s" s="0">
+      <c r="A27" t="s">
         <v>379</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B27" t="s">
         <v>380</v>
       </c>
-      <c r="C27" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D27" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E27" t="s" s="0">
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
         <v>381</v>
       </c>
-      <c r="F27" t="s" s="0">
+      <c r="F27" t="s">
         <v>382</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -4412,22 +4376,22 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s" s="0">
+      <c r="A28" t="s">
         <v>383</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B28" t="s">
         <v>384</v>
       </c>
-      <c r="C28" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D28" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E28" t="s" s="0">
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s">
         <v>385</v>
       </c>
-      <c r="F28" t="s" s="0">
+      <c r="F28" t="s">
         <v>386</v>
       </c>
       <c r="G28" s="4" t="s">
@@ -4435,22 +4399,22 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s" s="0">
+      <c r="A29" t="s">
         <v>387</v>
       </c>
-      <c r="B29" t="s" s="0">
+      <c r="B29" t="s">
         <v>388</v>
       </c>
-      <c r="C29" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D29" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E29" t="s" s="0">
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
         <v>389</v>
       </c>
-      <c r="F29" t="s" s="0">
+      <c r="F29" t="s">
         <v>390</v>
       </c>
       <c r="G29" s="4" t="s">
@@ -4458,646 +4422,646 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s" s="0">
+      <c r="A30" t="s">
         <v>391</v>
       </c>
-      <c r="B30" t="s" s="0">
+      <c r="B30" t="s">
         <v>392</v>
       </c>
-      <c r="C30" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D30" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E30" t="s" s="0">
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s">
         <v>393</v>
       </c>
-      <c r="F30" t="s" s="0">
+      <c r="F30" t="s">
         <v>394</v>
       </c>
-      <c r="G30" t="s" s="0">
+      <c r="G30" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" t="s" s="0">
+      <c r="A31" t="s">
         <v>395</v>
       </c>
-      <c r="B31" t="s" s="0">
+      <c r="B31" t="s">
         <v>396</v>
       </c>
-      <c r="C31" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D31" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E31" t="s" s="0">
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
         <v>45</v>
       </c>
-      <c r="F31" t="s" s="0">
+      <c r="F31" t="s">
         <v>397</v>
       </c>
-      <c r="G31" t="s" s="0">
+      <c r="G31" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" t="s" s="0">
+      <c r="A32" t="s">
         <v>398</v>
       </c>
-      <c r="B32" t="s" s="0">
+      <c r="B32" t="s">
         <v>399</v>
       </c>
-      <c r="C32" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D32" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E32" t="s" s="0">
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" t="s">
         <v>51</v>
       </c>
-      <c r="F32" t="s" s="0">
+      <c r="F32" t="s">
         <v>400</v>
       </c>
-      <c r="G32" t="s" s="0">
+      <c r="G32" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s" s="0">
+      <c r="A33" t="s">
         <v>401</v>
       </c>
-      <c r="B33" t="s" s="0">
+      <c r="B33" t="s">
         <v>402</v>
       </c>
-      <c r="C33" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D33" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E33" t="s" s="0">
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s">
         <v>63</v>
       </c>
-      <c r="F33" t="s" s="0">
+      <c r="F33" t="s">
         <v>403</v>
       </c>
-      <c r="G33" t="s" s="0">
+      <c r="G33" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s" s="0">
+      <c r="A34" t="s">
         <v>404</v>
       </c>
-      <c r="B34" t="s" s="0">
+      <c r="B34" t="s">
         <v>405</v>
       </c>
-      <c r="C34" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D34" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E34" t="s" s="0">
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" t="s">
         <v>69</v>
       </c>
-      <c r="F34" t="s" s="0">
+      <c r="F34" t="s">
         <v>406</v>
       </c>
-      <c r="G34" t="s" s="0">
+      <c r="G34" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s" s="0">
+      <c r="A35" t="s">
         <v>407</v>
       </c>
-      <c r="B35" t="s" s="0">
+      <c r="B35" t="s">
         <v>408</v>
       </c>
-      <c r="C35" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D35" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E35" t="s" s="0">
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
         <v>409</v>
       </c>
-      <c r="F35" t="s" s="0">
+      <c r="F35" t="s">
         <v>410</v>
       </c>
-      <c r="G35" t="s" s="0">
+      <c r="G35" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s" s="0">
+      <c r="A36" t="s">
         <v>411</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B36" t="s">
         <v>412</v>
       </c>
-      <c r="C36" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D36" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E36" t="s" s="0">
+      <c r="C36" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
         <v>413</v>
       </c>
-      <c r="F36" t="s" s="0">
+      <c r="F36" t="s">
         <v>414</v>
       </c>
-      <c r="G36" t="s" s="0">
+      <c r="G36" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s" s="0">
+      <c r="A37" t="s">
         <v>415</v>
       </c>
-      <c r="B37" t="s" s="0">
+      <c r="B37" t="s">
         <v>416</v>
       </c>
-      <c r="C37" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D37" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E37" t="s" s="0">
+      <c r="C37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" t="s">
         <v>413</v>
       </c>
-      <c r="F37" t="s" s="0">
+      <c r="F37" t="s">
         <v>414</v>
       </c>
-      <c r="G37" t="s" s="0">
+      <c r="G37" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" t="s" s="0">
+      <c r="A38" t="s">
         <v>417</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B38" t="s">
         <v>418</v>
       </c>
-      <c r="C38" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D38" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E38" t="s" s="0">
+      <c r="C38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" t="s">
         <v>419</v>
       </c>
-      <c r="F38" t="s" s="0">
+      <c r="F38" t="s">
         <v>420</v>
       </c>
-      <c r="G38" t="s" s="0">
+      <c r="G38" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" t="s" s="0">
+      <c r="A39" t="s">
         <v>421</v>
       </c>
-      <c r="B39" t="s" s="0">
+      <c r="B39" t="s">
         <v>422</v>
       </c>
-      <c r="C39" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D39" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E39" t="s" s="0">
+      <c r="C39" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
         <v>423</v>
       </c>
-      <c r="F39" t="s" s="0">
+      <c r="F39" t="s">
         <v>424</v>
       </c>
-      <c r="G39" t="s" s="0">
+      <c r="G39" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" t="s" s="0">
+      <c r="A40" t="s">
         <v>425</v>
       </c>
-      <c r="B40" t="s" s="0">
+      <c r="B40" t="s">
         <v>426</v>
       </c>
-      <c r="C40" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D40" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E40" t="s" s="0">
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" t="s">
         <v>427</v>
       </c>
-      <c r="F40" t="s" s="0">
+      <c r="F40" t="s">
         <v>428</v>
       </c>
-      <c r="G40" t="s" s="0">
+      <c r="G40" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" t="s" s="0">
+      <c r="A41" t="s">
         <v>429</v>
       </c>
-      <c r="B41" t="s" s="0">
+      <c r="B41" t="s">
         <v>430</v>
       </c>
-      <c r="C41" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D41" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E41" t="s" s="0">
+      <c r="C41" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s">
         <v>431</v>
       </c>
-      <c r="F41" t="s" s="0">
+      <c r="F41" t="s">
         <v>432</v>
       </c>
-      <c r="G41" t="s" s="0">
+      <c r="G41" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s" s="0">
+      <c r="A42" t="s">
         <v>433</v>
       </c>
-      <c r="B42" t="s" s="0">
+      <c r="B42" t="s">
         <v>434</v>
       </c>
-      <c r="C42" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E42" t="s" s="0">
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" t="s">
         <v>435</v>
       </c>
-      <c r="F42" t="s" s="0">
+      <c r="F42" t="s">
         <v>436</v>
       </c>
-      <c r="G42" t="s" s="0">
+      <c r="G42" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s" s="0">
+      <c r="A43" t="s">
         <v>437</v>
       </c>
-      <c r="B43" t="s" s="0">
+      <c r="B43" t="s">
         <v>438</v>
       </c>
-      <c r="C43" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D43" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E43" t="s" s="0">
+      <c r="C43" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s">
         <v>439</v>
       </c>
-      <c r="F43" t="s" s="0">
+      <c r="F43" t="s">
         <v>440</v>
       </c>
-      <c r="G43" t="s" s="0">
+      <c r="G43" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" t="s" s="0">
+      <c r="A44" t="s">
         <v>441</v>
       </c>
-      <c r="B44" t="s" s="0">
+      <c r="B44" t="s">
         <v>442</v>
       </c>
-      <c r="C44" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D44" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E44" t="s" s="0">
+      <c r="C44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" t="s">
         <v>443</v>
       </c>
-      <c r="F44" t="s" s="0">
+      <c r="F44" t="s">
         <v>444</v>
       </c>
-      <c r="G44" t="s" s="0">
+      <c r="G44" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="s" s="0">
+      <c r="A45" t="s">
         <v>447</v>
       </c>
-      <c r="B45" t="s" s="0">
+      <c r="B45" t="s">
         <v>448</v>
       </c>
-      <c r="C45" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D45" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E45" t="s" s="0">
+      <c r="C45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" t="s">
         <v>449</v>
       </c>
-      <c r="F45" t="s" s="0">
+      <c r="F45" t="s">
         <v>450</v>
       </c>
-      <c r="G45" t="s" s="0">
+      <c r="G45" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="s" s="0">
+      <c r="A46" t="s">
         <v>451</v>
       </c>
-      <c r="B46" t="s" s="0">
+      <c r="B46" t="s">
         <v>452</v>
       </c>
-      <c r="C46" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D46" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E46" t="s" s="0">
+      <c r="C46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
         <v>453</v>
       </c>
-      <c r="F46" t="s" s="0">
+      <c r="F46" t="s">
         <v>454</v>
       </c>
-      <c r="G46" t="s" s="0">
+      <c r="G46" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" t="s" s="0">
+      <c r="A47" t="s">
         <v>455</v>
       </c>
-      <c r="B47" t="s" s="0">
+      <c r="B47" t="s">
         <v>456</v>
       </c>
-      <c r="C47" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D47" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E47" t="s" s="0">
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s">
         <v>457</v>
       </c>
-      <c r="F47" t="s" s="0">
+      <c r="F47" t="s">
         <v>458</v>
       </c>
-      <c r="G47" t="s" s="0">
+      <c r="G47" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" t="s" s="0">
+      <c r="A48" t="s">
         <v>445</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B48" t="s">
         <v>446</v>
       </c>
-      <c r="C48" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E48" t="s" s="0">
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" t="s">
         <v>443</v>
       </c>
-      <c r="F48" t="s" s="0">
+      <c r="F48" t="s">
         <v>444</v>
       </c>
-      <c r="G48" t="s" s="0">
+      <c r="G48" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" t="s" s="0">
+      <c r="A49" t="s">
         <v>459</v>
       </c>
-      <c r="B49" t="s" s="0">
+      <c r="B49" t="s">
         <v>460</v>
       </c>
-      <c r="C49" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D49" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E49" t="s" s="0">
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s">
         <v>461</v>
       </c>
-      <c r="F49" t="s" s="0">
+      <c r="F49" t="s">
         <v>462</v>
       </c>
-      <c r="G49" t="s" s="0">
+      <c r="G49" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" t="s" s="0">
+      <c r="A50" t="s">
         <v>463</v>
       </c>
-      <c r="B50" t="s" s="0">
+      <c r="B50" t="s">
         <v>464</v>
       </c>
-      <c r="C50" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D50" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E50" t="s" s="0">
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s">
         <v>465</v>
       </c>
-      <c r="F50" t="s" s="0">
+      <c r="F50" t="s">
         <v>466</v>
       </c>
-      <c r="G50" t="s" s="0">
+      <c r="G50" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" t="s" s="0">
+      <c r="A51" t="s">
         <v>467</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B51" t="s">
         <v>468</v>
       </c>
-      <c r="C51" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D51" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E51" t="s" s="0">
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s">
         <v>465</v>
       </c>
-      <c r="F51" t="s" s="0">
+      <c r="F51" t="s">
         <v>466</v>
       </c>
-      <c r="G51" t="s" s="0">
+      <c r="G51" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s" s="0">
+      <c r="A52" t="s">
         <v>469</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B52" t="s">
         <v>470</v>
       </c>
-      <c r="C52" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D52" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E52" t="s" s="0">
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
         <v>471</v>
       </c>
-      <c r="F52" t="s" s="0">
+      <c r="F52" t="s">
         <v>472</v>
       </c>
-      <c r="G52" t="s" s="0">
+      <c r="G52" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s" s="0">
+      <c r="A53" t="s">
         <v>473</v>
       </c>
-      <c r="B53" t="s" s="0">
+      <c r="B53" t="s">
         <v>474</v>
       </c>
-      <c r="C53" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D53" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E53" t="s" s="0">
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
         <v>471</v>
       </c>
-      <c r="F53" t="s" s="0">
+      <c r="F53" t="s">
         <v>472</v>
       </c>
-      <c r="G53" t="s" s="0">
+      <c r="G53" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" t="s" s="0">
+      <c r="A54" t="s">
         <v>475</v>
       </c>
-      <c r="B54" t="s" s="0">
+      <c r="B54" t="s">
         <v>476</v>
       </c>
-      <c r="C54" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D54" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E54" t="s" s="0">
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" t="s">
         <v>477</v>
       </c>
-      <c r="F54" t="s" s="0">
+      <c r="F54" t="s">
         <v>478</v>
       </c>
-      <c r="G54" t="s" s="0">
+      <c r="G54" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s" s="0">
+      <c r="A55" t="s">
         <v>479</v>
       </c>
-      <c r="B55" t="s" s="0">
+      <c r="B55" t="s">
         <v>480</v>
       </c>
-      <c r="C55" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D55" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E55" t="s" s="0">
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
         <v>481</v>
       </c>
-      <c r="F55" t="s" s="0">
+      <c r="F55" t="s">
         <v>482</v>
       </c>
-      <c r="G55" t="s" s="0">
+      <c r="G55" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s" s="0">
+      <c r="A56" t="s">
         <v>483</v>
       </c>
-      <c r="B56" t="s" s="0">
+      <c r="B56" t="s">
         <v>484</v>
       </c>
-      <c r="C56" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D56" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E56" t="s" s="0">
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" t="s">
         <v>485</v>
       </c>
-      <c r="F56" t="s" s="0">
+      <c r="F56" t="s">
         <v>486</v>
       </c>
-      <c r="G56" t="s" s="0">
+      <c r="G56" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s" s="0">
+      <c r="A57" t="s">
         <v>487</v>
       </c>
-      <c r="B57" t="s" s="0">
+      <c r="B57" t="s">
         <v>488</v>
       </c>
-      <c r="C57" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="D57" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="E57" t="s" s="0">
+      <c r="C57" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
         <v>489</v>
       </c>
-      <c r="F57" t="s" s="0">
+      <c r="F57" t="s">
         <v>490</v>
       </c>
-      <c r="G57" t="s" s="0">
+      <c r="G57" t="s">
         <v>13</v>
       </c>
     </row>
@@ -5110,37 +5074,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s" s="0">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
improve report and count process
</commit_message>
<xml_diff>
--- a/src/main/resources/resultados_aprobaciones.xlsx
+++ b/src/main/resources/resultados_aprobaciones.xlsx
@@ -47,13 +47,18 @@
     <sheet name="resultados_27_03_26_13_59" r:id="rId35" sheetId="39"/>
     <sheet name="resultados_27_03_26_14_20" r:id="rId36" sheetId="40"/>
     <sheet name="resultados_27_03_26_21_25" r:id="rId37" sheetId="41"/>
+    <sheet name="resultados_27_03_26_21_39" r:id="rId38" sheetId="42"/>
+    <sheet name="resultados_27_03_26_21_44" r:id="rId39" sheetId="43"/>
+    <sheet name="resultados_27_03_26_21_47" r:id="rId40" sheetId="44"/>
+    <sheet name="resultados_30_03_26_10_32" r:id="rId41" sheetId="45"/>
+    <sheet name="resultados_30_03_26_17_05" r:id="rId42" sheetId="46"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9632" uniqueCount="4471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10262" uniqueCount="4747">
   <si>
     <t>Referencia</t>
   </si>
@@ -13466,6 +13471,834 @@
   </si>
   <si>
     <t>27/03/2026 05:30 p. m.</t>
+  </si>
+  <si>
+    <t>CF83A856-5F95-435D-87A0-A0C64A7DEA34</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: SOLICITUD REVOCATORIA SANCIÓN-HECHO SUPERADO INSTANCIA: FALLO SANCIÓN REFERENCIA:ACCIÓN DE TUTELA RADICADO: 180013104001202500086 ACCIONANTE: MARÍA PATRICIA DÍAZ VARGAS ACCIONADO: SECRETARÍA DE EDUCACIÓN DEL CAQUETÁ Y FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO ORIÓN: 314205</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:11 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:11 a. m.</t>
+  </si>
+  <si>
+    <t>D47FDB27-1773-4BF3-B158-9BDBA04BF95E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: NUEVO ALCANCE- INAPLICACIÓN INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 13-001-31-07-003-2026-0004-00 ACCIONANTE: MARÍA TERESA JARAMILLO NIÑO ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORIÓN: 313992</t>
+  </si>
+  <si>
+    <t>30/03/2026 09:36 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 10:36 a. m.</t>
+  </si>
+  <si>
+    <t>BCA9F824-C325-47C3-AD76-EA70A725E550</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: SOLICITUD DE INAPLICACIÓN SANCIÓN-HECHO SUPERADO INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO:110013109009 2025-00331 ACCIONANTE: JAVIER SANTACRUZ PONCE como apoderado de CLARA ÁVILA DE MARTÍNEZ ACCIONADO: FIDUPREVISORA S.A. ORIÓN:302429</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:14 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:14 a. m.</t>
+  </si>
+  <si>
+    <t>58984BE2-EC06-44CA-BB61-FDF3871E6A8B</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 23162310400120260000300 ACCIONANTE: MARÍA MIRIAM SÁNCHEZ PAEZ ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 314034</t>
+  </si>
+  <si>
+    <t>30/03/2026 09:29 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 10:29 a. m.</t>
+  </si>
+  <si>
+    <t>92214729-A32C-47EF-B48E-B8A150260EF0</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE INAPLICACION Y/O INEJECUCIÓN INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 17001311000520260004800 ACCIONANTE: LUZ ESTELA GIRALDO LEIVA ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313885</t>
+  </si>
+  <si>
+    <t>30/03/2026 09:28 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 10:28 a. m.</t>
+  </si>
+  <si>
+    <t>0F5A6B52-6E25-479A-8EB5-D54128AD5D5F</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME IMPUGNACIÓN RADICADO: 47001-31-60-004-2026-00089-00 ACCIONANTE: ROSA MARÍA TORRES OSPINO ACCIONADO: FOMAG ORIÓN: 313988</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:24 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:24 a. m.</t>
+  </si>
+  <si>
+    <t>ECA2E70F-8EEE-4A2D-822F-4D0A907CCAA2</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE INAPLICACION - INEJECUCIÓN - NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 73001333300520250030200 ACCIONANTE: LAURA OSORIO MOLINA AGENTE OFICIOSA DE ELOISA MOLINA ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313861</t>
+  </si>
+  <si>
+    <t>30/03/2026 09:26 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 10:26 a. m.</t>
+  </si>
+  <si>
+    <t>783775C9-5563-4977-B5ED-9CAA57B2CF1F</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 2026 00038 ACCIONANTE: OSCAR VILLALBA PATERNINA. ACCIONADO: FOMAG ORIÓN: 313591</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:30 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:30 a. m.</t>
+  </si>
+  <si>
+    <t>001E6AB7-06FE-4BC8-871E-3D6BE16FBCC4</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD E INAPLICACIÓN INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 11001310504620251021700 ACCIONANTE: DAVID ENRIQUE GALLO DURANGO ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 312651</t>
+  </si>
+  <si>
+    <t>30/03/2026 09:19 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 10:19 a. m.</t>
+  </si>
+  <si>
+    <t>50CF802A-2482-41B6-85FC-37E65BB0F3E6</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INCIDENTE DE DESCATO RADICADO: 17001333900820250038800 ACCIONANTE: ALBA LUCÍA MARÍN CARDONA ACCIONADO: FIDUPREVISORA – FOMAG ORIÓN: 306700</t>
+  </si>
+  <si>
+    <t>29/03/2026 11:34 p. m.</t>
+  </si>
+  <si>
+    <t>95C9728D-DADA-49C2-9F16-9C14FC373E9E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: CUMPLIMIENTO DE FALLO RADICADO: 08001310501520261000800 ACCIONANTE: JESUS ESTEBAN PALACIO IMPARATO ACCIONADO: FIDUPREVISORA – FOMAG ORION: 309920</t>
+  </si>
+  <si>
+    <t>29/03/2026 11:33 p. m.</t>
+  </si>
+  <si>
+    <t>997F0D8F-0494-43A3-B73A-BB7E1A4357AD</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REF. CONTESTACIÓN ACCIÓN DE TUTELA ACCIONANTE: LUIS HILDEBRANDO CRUZ BARÓN ACCIONADOFONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG; FIDUPREVISORA S.A RADICADO: 15806-40-89-001-2026-00031-00 ORIÓN:308237</t>
+  </si>
+  <si>
+    <t>07BC3A3B-D869-46CB-89EC-2A21EED68AFE</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME RADICADO: 470014189005202300731 ACCIONANTE: JERLIS JASMIN GONZALEZ COLLAZOS, en representación de su menor hijo ENZHO FARITH SALCEDO ACCIONADO: FONDO NACIONAL DE PRESTACIONES DEL MAGISTERIO y FIDUPREVISO-RA ORIÓN: 311586</t>
+  </si>
+  <si>
+    <t>29/03/2026 09:01 p. m.</t>
+  </si>
+  <si>
+    <t>7B062CBF-FEDE-4B18-9A07-0CFFF9DE3B05</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 23-001-41-05-001-2025-10379-00 ACCIONANTE: ANA MILENA VARELA PADILLA ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314202</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:37 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:37 a. m.</t>
+  </si>
+  <si>
+    <t>3B930070-9924-41AA-BC21-79082B32F2C5</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 05736318400120260001000 ACCIONANTE: BEATRIZ YAMILE MARÍN TILANO ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313934</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:35 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:35 a. m.</t>
+  </si>
+  <si>
+    <t>0B6B2649-2DD8-47DF-B62E-5F1D67C5E5A0</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 23570408900120250047000 ACCIONANTE: MARIO MIGUEL MUÑOZ MARQUEZ ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313425</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:34 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:34 a. m.</t>
+  </si>
+  <si>
+    <t>FB1E852A-0D77-4D64-BF5E-D4396CBAE879</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 05284318400120260000500 ACCIONANTE: HERNÁN DE JESÚS HURTADO ARIAS ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313906</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:33 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:33 a. m.</t>
+  </si>
+  <si>
+    <t>C5A077A2-049C-44F1-B3B3-99505C215FCD</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 05001333300220260006900 ACCIONANTE: MARTHA NELLY MARÍN MARÍN. ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 313331</t>
+  </si>
+  <si>
+    <t>30/03/2026 10:31 a. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 11:31 a. m.</t>
+  </si>
+  <si>
+    <t>E8988326-4C24-4982-95A3-12A0F71051B4</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 05579 31 84 001 2026 00059 00. ACCIONANTE: OSCAR JAUREGUI GELVES ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 313657</t>
+  </si>
+  <si>
+    <t>045E798F-CAE2-40A6-84CC-2E4C2C2850A1</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 05.001.31.87.006.2026.00065.00. ACCIONANTE: SANDRA MILENA CANO RUÍZ ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 313602</t>
+  </si>
+  <si>
+    <t>43354568-4C60-42D1-952D-0CD5A2EF4F57</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: PROCESO: INCIDENTE DESACATO RADICACIÓN: 08001-31-05-010-2025-10135-00 INCIDENTANTE: NELLY CALVO ESCOBAR INCIDENTADO: FIDUPREVISORA S.A. – DIRECCIÓN DE PRESTACIONES ECONÓMICAS ORION: 312655</t>
+  </si>
+  <si>
+    <t>27BDADE2-8B31-46B1-9896-88F5E16D6B31</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 47001310700320250004800 ACCIONANTE: LINA PATRICIA JIMENO VALDERRAMA ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 307795</t>
+  </si>
+  <si>
+    <t>E8726EF2-F4CA-4947-ADDB-8D243E72E653</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: RESPUESTA REQUERIMIENTO REFERENCIA: REQUERIMIENTO RADICADO: 050013187003202500242 ACCIONANTE: ISABEL BEATRIZ DE JESUS SAMPAYO NEGRETTE ACCIONADO: FIDUPREVISORA - FOMAG ORION: 314161</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:47 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:47 p. m.</t>
+  </si>
+  <si>
+    <t>9BD94808-5395-4154-AAC4-CF9792B865E0</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE CUMPLIMIENTO RADICADO: 11001-318701620250005300 ACCIONANTE: MARIA DEL ROSARIO BARRAZA LOZANO ACCIONADO: FIDUPREVISORA -FOMAG ORIÓN: 310367</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:48 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:48 p. m.</t>
+  </si>
+  <si>
+    <t>00637BAE-204B-4A16-B1D7-0F395147BC7A</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 08-001-33-33-013-2025-00184-00 ACCIONANTE: CECILIO ANTONIO ROMERO DE LA HOZ ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314406</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:46 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:46 p. m.</t>
+  </si>
+  <si>
+    <t>B600F7B2-6717-4687-B0E0-1CBCAAC4319B</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME FALLO DE ACCIÓN DE TUTELA RADICADO: 2026-00007 ACCIONANTE: MARIELINA MELO MARTÍNEZ C.C. 23693960 ACCIONADO: FIDUPREVISORA S.A. ORIÓN: 313293</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:06 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:06 p. m.</t>
+  </si>
+  <si>
+    <t>197E2B92-C466-485E-810E-76242EB8367A</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: IMPUGNACION REFERENCIA ACCION DE TUTELA RADICADO: 050013 0502720261004600 ACCIONANTE: ORLANDO ANTONIO SILVA RAMOS ACCIONADO: FIDUPREVISORA S.A. – FOMAG – SECRETARIA DE EDUCACIÓN ORIÓN: 313705</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:08 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 05:08 p. m.</t>
+  </si>
+  <si>
+    <t>8A017A7D-7673-478E-BFF4-0D5624052509</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: OFICIO DE GESTION RADICADO TUTELA: 66001-31-18-001-2026-00027-00 ACCIONANTE: JOSÉ BERSEIN GONZÁLEZ PÁEZ ACCIONADO: FIDUPREVISORA S.A y OTROS ORIÓN: 314079</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:59 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:59 p. m.</t>
+  </si>
+  <si>
+    <t>EB62FAF0-095D-46BB-A84E-1648E502055E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 150013109002202600002-00 ACCIONANTE: ELMER ASDRÚBAL GÓMEZ VILLATE ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314413</t>
+  </si>
+  <si>
+    <t>E4A1E9A3-34B9-445B-8A39-2B95876D3E51</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD REFERENCIA: FALLO DE PRIMERA INSTANCIA REFERENCIA: 23 660 31 84 001 2026 00053 00 ACCIONANTE: FRANCISCO TOMAS RIVERO RUIZ ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314430</t>
+  </si>
+  <si>
+    <t>92171626-6242-486A-8E3F-8F1C7279F5DF</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 2026.00021.01 ACCIONANTE: ROBINSON JOSE MULFORD LEYVA ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314208</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:58 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:58 p. m.</t>
+  </si>
+  <si>
+    <t>5D3F59B6-424F-4057-83C7-705D333A3F49</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE CUMPLIMIENTO RADICADO: 05 001 31 87 011 2026 00002 01. ACCIONANTE: SAMUEL GIRALDO ZULUAGA ACCIONADO: FONDO DE PRESTACIONES DEL MAGISTERIO- FOMAG Y OTROS ORIÓN: 305752</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:57 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:57 p. m.</t>
+  </si>
+  <si>
+    <t>A65DF6BC-E553-4F07-99CC-2C33DD44CBC8</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 202601336 DANIEL GONZALEZ RAYO</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:56 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:56 p. m.</t>
+  </si>
+  <si>
+    <t>3DE4B600-6A39-4A51-BE34-DA186D958C1E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 2026-01019 HENRY BAEZA ARAGON</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:55 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:55 p. m.</t>
+  </si>
+  <si>
+    <t>191A11B5-9FD7-43F9-A336-F332BB667420</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 2026-00051 ALBA ROSA MENDIVELSO</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:54 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:54 p. m.</t>
+  </si>
+  <si>
+    <t>E025B725-7DD2-417C-B888-7E768AAFE4F7</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: CUMPLIMIENTO A FALLO. RADICADO: 110013403-004-2026-00044-00 ACCIONANTE: FABIO LUIS GARCÍA MORALES ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 313769</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:17 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 05:17 p. m.</t>
+  </si>
+  <si>
+    <t>011EA433-BBF9-4EC5-BE31-8FD1DE4067CD</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN RADICACIÓN: 76-834-31-03-003-2025-00253-00 ACCIONANTE: EFRAIN TORRES CASTAÑEDA ACCIONADO: FIDUPREVISORA S.A. ORION: 308482</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:20 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 05:20 p. m.</t>
+  </si>
+  <si>
+    <t>52EC0CF0-E051-4CE7-ADFB-0695A1FC6E77</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE SUSPENSIÓN E INFORME DE GESTION INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 669001310900820250011800 ACCIONANTE: GABRIEL CANO RUIZ ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 313973</t>
+  </si>
+  <si>
+    <t>30/03/2026 03:53 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 04:53 p. m.</t>
+  </si>
+  <si>
+    <t>4FC06664-B4D3-4DDF-A023-4F7BA30CC943</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 41001310500220251012400 ACCIONANTE: ALBA MERCEDES CARDENAS CEDEÑO ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314218</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:35 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:35 a. m.</t>
+  </si>
+  <si>
+    <t>C53FC37D-176B-4240-938C-11C26626C5D0</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: RESPUESTA REQUERIMIENTO REFERENCIA: REQUERIMIENTO RADICADO: 05001333301420250043400 ACCIONANTE: DIANA ALEXANDRA ZULUAGA ROMAN ACCIONADO: FIDUPREVISORA - FOMAG ORION: 312323</t>
+  </si>
+  <si>
+    <t>F4A45A6B-898D-47B0-9039-43135362932C</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 05001-40-09-034-2025-00368 ACCIONANTE: LUZ MERY PARRA HOYOS en representación de LIZETH JOHANA LOPÉZ PARRA ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 312833</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:39 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:39 a. m.</t>
+  </si>
+  <si>
+    <t>FE34B535-A985-4429-90D8-3E4DCFBB35EA</t>
+  </si>
+  <si>
+    <t>1A9E8895-3683-4980-B7E0-E1A182840863</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 2026-10016 ALCIRA BEATRIZ RUBIANO GAITAN</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:42 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:42 a. m.</t>
+  </si>
+  <si>
+    <t>67314E98-8526-432E-BA17-8DDB4DEC7676</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 05001400300920150116100 ACCIONANTE: ALBA LUZ MAZO GIRALDO ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORION: 314523</t>
+  </si>
+  <si>
+    <t>8B48776D-BE4E-4EEB-8BAA-1CAB63929F47</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 050013103014202600054 ACCIONANTE: MARIA DE JESUS SANCHEZ MARÍN ACCIONADO: FOMAG-FIDUPREVISORA ORION: 313228</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:34 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:34 a. m.</t>
+  </si>
+  <si>
+    <t>D6E02228-5895-4B2D-90D1-C3D9CD2158B8</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: CONTESTACIÓN REFERENCIA: INFORME DE GESTIÓN E IMPOSIBILIDAD JURIDICA RADICACIÓN: 76147333300420250021600 ACCIONANTE: MARÍA EDITH CARDONA MORALES ACCIONADO: DEPARTAMENTO DEL VALLE DEL CAUCA – SECRETARÍA DE EDUCACIÓN FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO - FOMAG ORION: 308546</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:22 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 05:22 p. m.</t>
+  </si>
+  <si>
+    <t>D060BEB3-51D4-43F3-AE3E-B8701A2C2391</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN RADICACIÓN: 0561531040022026-00024 ACCIONANTE: Jaime Alberto Arcila Quintero ACCIONADO: Fiduprevisora S.A., en calidad de vocera y administradora del Patrimonio Autó-nomo Fondo Nacional de Prestaciones Sociales del Magisterio – Fomag ORION: 311715</t>
+  </si>
+  <si>
+    <t>9C328300-9A48-4A57-B4FB-2ED0DD46ACC3</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME FALLO DE ACCIÓN DE TUTELA RADICADO: 2025-00216 ACCIONANTE: HERNANDO VERGARA PINZON C.C. 79694188 ACCIONADO: FIDUPREVISORA S.A. Y FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO ORIÓN: 314060</t>
+  </si>
+  <si>
+    <t>463A2D30-FB51-4361-A7E3-D1E29F639A2E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN RADICACIÓN: 47-001-3333-012-2026-00023-00 ACCIONANTE: JULIO CESAR TORRES MONTENEGRO ACCIONADO: Dirección de Prestaciones Económicas – Fondo Nacional de Prestaciones Sociales del Magisterio, Fomag – Fiduprevisora S.A ORION: 310644</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:21 p. m.</t>
+  </si>
+  <si>
+    <t>31/03/2026 05:21 p. m.</t>
+  </si>
+  <si>
+    <t>67678701-2BCC-424F-9991-62231C303786</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 2026-00012 MARIA DEL SOCORRO DURANGO JARAMILLO</t>
+  </si>
+  <si>
+    <t>830922F8-33D7-4F70-AE60-74272DFE17F7</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN RADICACIÓN: 23-001-33-33-001-2025-00304-00 ACCIONANTE: MARY LUZ CANTERO HOYOS ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO Y SECRETARÍA DE EDUCACIÓN DE CÓRDOBA ORION: 308602</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:44 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:44 a. m.</t>
+  </si>
+  <si>
+    <t>0F355CD6-6D07-4130-9674-B79F02DE9077</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE CUMPLIMIENTO RADICADO: 760013110006-2020-00266-20 ACCIONANTE: JORGE LUIS RAMOS SOLARTE ACCIONADO: Fondo Nacional de Prestaciones Sociales del Magisterio - FOMAG ORIÓN: 307008</t>
+  </si>
+  <si>
+    <t>FCE310A8-2954-498A-9CAF-6760ACC1B1F4</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN RADICACIÓN: 2026-00011 ACCIONANTE: MYRIAM QUINTERO PARIAS ACCIONADO: Secretaría de Educación Municipal de Armenia, Fondo de Prestaciones Sociales del Magisterio del Departamento del Quindío y Fiduprevisora S.A., ORION: 306897</t>
+  </si>
+  <si>
+    <t>BAF517CD-0A69-4631-8C4D-096EB4F25BDA</t>
+  </si>
+  <si>
+    <t>A183C8A5-9FF0-4D8D-93B0-544EBCB4860E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 170014003002-2022-00049-00 ACCIONANTE: NORA YANETH OCAMPO DUQUE ACCIONADO: COSMITET EPS ORIÓN: 312154</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:52 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:52 a. m.</t>
+  </si>
+  <si>
+    <t>A16B32F1-ECF0-4F85-A4B9-BA3A38A9966E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE CUMPLIMIENTO RADICADO: 23-162-31-84-001-2026-00019-00 ACCIONANTE: FAUSTINA CARO GARCÍA A/O JOSE DOLORES CARO ACCIONADO: Fondo Nacional de Prestaciones Sociales del Magisterio - FOMAG ORIÓN: 311634</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:51 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:51 a. m.</t>
+  </si>
+  <si>
+    <t>1EECB971-CE4A-436C-A50E-A55ADD6D33B5</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 680813104005-2025-00035-00 ACCIONANTE: SANDRA ISABEL SARMIENTO DIAZ ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO– FOMAG ORIÓN: 295291</t>
+  </si>
+  <si>
+    <t>5F04CC02-6129-473E-9E54-ECBD0FD1574C</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 050013103009 2024 00161 00 ACCIONANTE: PAULA ANDREA MONSALVE PÉREZ AFECTADO: LUIS MATEO RIVAS MONSALVE ACCIONADO: FIDUPREVISORA S.A COMO VOCERA Y ADMINISTRADORA DEL FOMAG ORIÓN: 312551</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:50 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:50 a. m.</t>
+  </si>
+  <si>
+    <t>FCE7B868-FFC2-4910-A90F-F793E605AF7A</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 08001333301120250023600 ACCIONANTE: MINERVA ISABEL DE LA HOZ DE VILLAMIZAR ACCIONADO: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG – FIDUPREVISORA – MINISTERIO DE EDUCACIÓN NACIONAL ORION: 310439</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:49 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:49 a. m.</t>
+  </si>
+  <si>
+    <t>F7CD82F9-027B-4E3B-AE7F-CCF69C3C1F47</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME DE GESTIÓN. RADICADO: 11001408807320202600078 ACCIONANTE: AURA MARÍA GUEVARA DE ESTUPIÑÁN ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO- FOMAG ORIÓN: 314022</t>
+  </si>
+  <si>
+    <t>A0CF45EF-6C6D-4B34-852C-4884E6BA1FB9</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 63001-3333-003-2025-00147-00 ACCIONANTE: DEYANIRA CEBALLOS DE FORERO ACCIONADO: NACIÓN – MINISTERIO DE EDUCACIÓN – FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO ORIÓN: 294966</t>
+  </si>
+  <si>
+    <t>A3F3D197-FAA3-4667-9A9D-C7FDF6EFD67C</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: SOLICITUD DE NULIDAD SANCIÓN - ACCIÓN DE TUTELA RADICADO: 05 697 31 12 001 2025-00253-00 ACCIONANTE: LUZ MERY CONDE CASTRILLÓN ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO (FOMAG)-FIDUPREVISORA ORION: 307132, 309414 y 313069</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:48 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:48 a. m.</t>
+  </si>
+  <si>
+    <t>4E6A1476-A4F3-4DF6-9C4D-D7E558B17C2B</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: IMPUGNACION REFERENCIA ACCION DE TUTELA RADICADO: 05001333300920260008100 ACCIONANTE: MARTHA LUCIA TOBON GOMEZ ACCIONADO: FIDUPREVISORA S.A. – FOMAG – SECRETARIA DE EDUCACIÓN ORIÓN: 313364</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:46 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:46 a. m.</t>
+  </si>
+  <si>
+    <t>E30AEB34-05B1-41E5-9558-17B53D8883BF</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: 2026-00031 RUDY MARIANA URQUIJO ACEVEDO</t>
+  </si>
+  <si>
+    <t>B067561E-5A25-42DA-87CE-C15C3BC0CADC</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME REFERENCIA: ACCIÓN DE TUTELA No. 66400-31-89-001-2026-00037-00 ACCIONANTE: ROSMARINA ULCHUR PILLIMUE ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG; FIDU-PREVISORA S.A ORION: 307451</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:01 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:01 a. m.</t>
+  </si>
+  <si>
+    <t>A9C8197E-A7EB-41E1-B6D2-9D28301FD5FE</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME RADICADO: 68001-34-03-001-2026-00019-01 ACCIONANTE: OLGA LILIANA GOMEZ DURAN ACCIONADO: FIDUPREVISORA en calidad de la vocera y administradora del FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO - FOMAG ORION: 311844</t>
+  </si>
+  <si>
+    <t>66B46898-AC90-4FCB-B52C-D362BBDDCDE0</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:00 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:00 a. m.</t>
+  </si>
+  <si>
+    <t>5EEB314F-5A14-4BD8-A385-1C725DEDB92B</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 110013110037-2025-00561-00 ACCIONANTE: MARIA DEL CARMEN BELTRAN ORJUELA ACCIONADO: FIDUPREVISORA S.A. ORION: 307260</t>
+  </si>
+  <si>
+    <t>228ADD73-ADD4-4A16-9C97-857ABC2CF18F</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE INAPLICACIÓN INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: OLGA LILIANA GOMEZ DURAN ACCIONANTE: 68001-34-01-001-2026-00019-01 ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORIÓN: 313167</t>
+  </si>
+  <si>
+    <t>61107819-F21D-4B39-99A0-82FD60A52C2F</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 2025-00150-01 ACCIONANTE: MARIA JOSÉ MAESTRE AVILA ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORIÓN: 314347</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:59 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:59 a. m.</t>
+  </si>
+  <si>
+    <t>AB8678CB-5EE7-442B-B117-605289967990</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD E INAPLICACIÓN INSTANCIA: SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: ANDRÉS ANTONIO GONZÁLEZ RODRÍGUEZ ACCIONANTE: 2026-00001-00 ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORIÓN: 313031</t>
+  </si>
+  <si>
+    <t>CDDC495B-BE8D-4009-92EC-2C0A8280D437</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: SOLICITUD DE NULIDAD, INAPLICACIÓN DE LA SANCIÓN REFERENCIA: ACCIÓN DE TUTELA RADICADO: 76834310500220260002300 ACCIONANTE: LILIANA PÉREZ TAMAYO ACCIONADO: FIDUPREVISORA S.A. – FOMAG ORIÓN: 314338</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:58 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:58 a. m.</t>
+  </si>
+  <si>
+    <t>AA5CEE2B-B53B-4103-ACFE-7C3B060AA7C6</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 080014009022-2025-00343-01 ACCIONANTE: ASTRID DEL CARMEN CASTILLO GALLARDO AFECTADO: CARLOS ADRIAN ROMERO CASTILLO ACCIONADO: IPS ORGANIZACIÓN CLÍNICA GENERAL DEL NORTE ORION: 296181</t>
+  </si>
+  <si>
+    <t>30/03/2026 04:53 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 08:53 a. m.</t>
+  </si>
+  <si>
+    <t>AA8B0883-1DF0-4BFE-8E32-54FC184FB859</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 73-001-31-03-004-2025-00305-00 ACCIONANTE: GONZALO REYES MOSCOSO AFECTADO: HILDA LUCÍA FLÓREZ ARDILA ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO FOMAG. ORIÓN: 310623</t>
+  </si>
+  <si>
+    <t>A38B1887-A2FE-43FB-A19A-D5B41D9754C1</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 11001-31-03-049-2025-00588-00 ACCIONANTE: ANA MARÍA VELÁSQUEZ DE CRUZ ACCIONADO: FIDUPREVISORA S.A. ORIÓN: 312990</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:18 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:18 a. m.</t>
+  </si>
+  <si>
+    <t>5A1E9040-5193-452C-A08F-A1926B6A87EB</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 41001 31 20 001 2025 00176 ACCIONANTE: ELVIA ESPERANZA CASTRO TORRES ACCIONADO: FIDUCIARIA LA PREVISORA S.A. ORIÓN: 308740</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:17 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:17 a. m.</t>
+  </si>
+  <si>
+    <t>AE23FA9F-B128-4F26-B2A7-F3A0E977F625</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE CUMPLIMIENTO A FALLO RADICADO: 190013333004 2026 00022 00 ACCIONANTE: CARMEN ALICIA HIDALGO DE BENAVIDES ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG – FIDUPREVISORA ORIÓN: 307161</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:13 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:13 a. m.</t>
+  </si>
+  <si>
+    <t>091EC24C-AD78-4961-A8E0-09A1C39E5E68</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: ASUNTO: INFORME DE CUMPLIMIENTO Y RESPUESTA A DESACATO REFERENCIA: 2026-00006-00 ACCIONANTE: ROGER ENRIQUE PINZÓN GARCIA ACCIONADOS: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG ORION: 314354</t>
+  </si>
+  <si>
+    <t>D242093F-BF9E-480E-A476-A909E9168A3E</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: SOLICITUD PERDIDA DE EJECUCIÓN COBRO COACTIVO POR DESVINCULACIÓN DE LA SANCIONADA Referenciado: Expediente Cobro Coactivo No. 05001129000020260054900</t>
+  </si>
+  <si>
+    <t>AC555C55-4E9A-47AA-97C3-F63F07D08AFD</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME RADICADO: 760014003025201000071 ACCIONANTE: YOLANDA CASTRO QUINTERO, EN REPRESENTACIÓN DE SU HIJO MENOR LUIS EDUARDO CASTRO ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO – FOMAG – COHAN VINCULADOS: FIDUPREVISORA S.A. COMO VOCERA Y ADMINISTRADORA DEL PATRI-MONIO FOMAG ORIÓN: 309747</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:12 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:12 a. m.</t>
+  </si>
+  <si>
+    <t>E35A6A8D-8F7D-4AD0-A157-C0EE86CD5FE1</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN TUTELA RADICADO: 25-843-31-03-001-2026-00046-00 ACCIONANTE: SANDRA ESTELA SANTANA CORTÉS AFECTADO: ÁLVARO AUGUSTO BAQUERO SANTANA ACCIONADO: FIDUPREVISORA S.A. ORION: 307074</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:11 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:11 a. m.</t>
+  </si>
+  <si>
+    <t>576FEA7A-DF04-4B62-9029-4EC111CEF6B1</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME FALLO DE ACCIÓN DE TUTELA RADICADO: 2025-00104 ACCIONANTE: JOSÉ JULIÁN VERGARA LÓPEZ C.C. 18590374 ACCIONADO: FIDUPREVISORA S.A. y FONDO DE PRESTACIONES DEL MAGISTERIO -FOMAG ORIÓN: 313928</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:31 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:30 a. m.</t>
+  </si>
+  <si>
+    <t>9E2BA40C-200C-4D8C-A91F-22DDB9A86976</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: INFORME DE GESTIÓN CUMPLIMIENTO A FALLO RADICADO: 47001310700320250013600 ACCIONANTE: MARCELA PAOLA GAMERO CANDELARIO ACCIONADO: FIDUPREVISORA (FOMAG) Y LA CLÍNICA GENERAL DEL NORTE. ORION: 307372</t>
+  </si>
+  <si>
+    <t>A86764C1-8F70-4E3A-9CD3-469510082C86</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME FALLO DE ACCIÓN DE TUTELA RADICADO: 2025-00119 ACCIONANTE: YANETH LUCIA PEREZ ZARATE C.C. 23275342 ACCIONADO: FONDO NACIONAL DE PRESTACIONES SOCIALES DEL MAGISTERIO (FOMAG) y FIDUPREVISORA S.A. ORIÓN: 314880</t>
+  </si>
+  <si>
+    <t>30/03/2026 05:05 p. m.</t>
+  </si>
+  <si>
+    <t>01/04/2026 09:05 a. m.</t>
+  </si>
+  <si>
+    <t>A70DCE08-22EA-4DC5-A109-7E3A0FA26F98</t>
+  </si>
+  <si>
+    <t>Aprobar o modificar comunicación de salida con asunto: REFERENCIA: INFORME FALLO DE ACCIÓN DE TUTELA RADICADO: 2025-00109 ACCIONANTE: ALEXANDRA MARITZA LOPEZ NAVARRO C.C. 1044619336 ACCIONADO: FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO FOMAG FIDUPREVISORA ORIÓN: 314435</t>
   </si>
 </sst>
 </file>
@@ -40812,6 +41645,2126 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>4471</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4472</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>4473</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>4474</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4475</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4476</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>4477</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>4478</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>4479</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>4480</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>4481</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>4482</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>4483</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4484</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>4485</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>4486</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>4487</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4488</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>4489</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>4490</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>4491</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4492</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>4493</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>4494</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>4495</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4496</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>4497</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>4498</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>4499</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4500</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>4501</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>4502</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>4503</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4504</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>4505</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>4506</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>4507</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4508</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>4509</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>4445</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>4510</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4511</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>4512</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>4445</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>4513</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4514</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>4501</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>4502</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>4515</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4516</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>4517</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>4445</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>4518</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4519</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>4520</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>4521</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>4522</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4523</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>4524</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>4525</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>4526</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4527</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>4528</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>4529</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>4530</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4531</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>4532</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>4533</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>4534</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4535</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>4536</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>4537</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>4538</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4539</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>4536</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>4537</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>4540</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4541</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>4536</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>4537</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>4542</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4543</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>4536</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>4537</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>4544</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4545</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>4501</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>4502</v>
+      </c>
+      <c r="G23" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G64"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>4546</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4547</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>4548</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>4549</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4550</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4551</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>4552</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>4553</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>4554</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>4555</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>4556</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>4557</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>4558</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4559</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>4560</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>4561</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>4562</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4563</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>4564</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>4565</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>4566</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4567</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>4568</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>4569</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>4570</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4571</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>4568</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>4569</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>4572</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4573</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>4568</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>4569</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>4574</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4575</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>4576</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>4577</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>4578</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4579</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>4580</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>4581</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>4582</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4583</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>4584</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>4585</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>4586</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4587</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>4588</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>4589</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>4590</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4591</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>4592</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>4593</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>4594</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4595</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>4596</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>4597</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>4598</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4599</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>4600</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>4601</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>4602</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4603</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>4604</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>4605</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>4606</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4607</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>4608</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>4609</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>4610</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4611</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>4608</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>4609</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>4612</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4613</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>4614</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>4615</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>4616</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>1773</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>4600</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>4601</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>4617</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4618</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>4619</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>4620</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>4621</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4622</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>4614</v>
+      </c>
+      <c r="F23" t="s" s="0">
+        <v>4615</v>
+      </c>
+      <c r="G23" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>4623</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>4624</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>4625</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>4626</v>
+      </c>
+      <c r="G24" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>4627</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>4628</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>4629</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>4630</v>
+      </c>
+      <c r="G25" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>4631</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>4632</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>4629</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>4630</v>
+      </c>
+      <c r="G26" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>4633</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>4634</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>4629</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>4630</v>
+      </c>
+      <c r="G27" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>4635</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>4636</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>4637</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>4638</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>4639</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>4640</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>4619</v>
+      </c>
+      <c r="F29" t="s" s="0">
+        <v>4620</v>
+      </c>
+      <c r="G29" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>4641</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>4642</v>
+      </c>
+      <c r="C30" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>4643</v>
+      </c>
+      <c r="F30" t="s" s="0">
+        <v>4644</v>
+      </c>
+      <c r="G30" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>4645</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>4646</v>
+      </c>
+      <c r="C31" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>4637</v>
+      </c>
+      <c r="F31" t="s" s="0">
+        <v>4638</v>
+      </c>
+      <c r="G31" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>4647</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>4648</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>4637</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>4638</v>
+      </c>
+      <c r="G32" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>4649</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>4648</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>4600</v>
+      </c>
+      <c r="F33" t="s" s="0">
+        <v>4601</v>
+      </c>
+      <c r="G33" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>4650</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>4651</v>
+      </c>
+      <c r="C34" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E34" t="s" s="0">
+        <v>4652</v>
+      </c>
+      <c r="F34" t="s" s="0">
+        <v>4653</v>
+      </c>
+      <c r="G34" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>4654</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>4655</v>
+      </c>
+      <c r="C35" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s" s="0">
+        <v>4656</v>
+      </c>
+      <c r="F35" t="s" s="0">
+        <v>4657</v>
+      </c>
+      <c r="G35" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>4658</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>4659</v>
+      </c>
+      <c r="C36" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>4656</v>
+      </c>
+      <c r="F36" t="s" s="0">
+        <v>4657</v>
+      </c>
+      <c r="G36" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>4660</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>4661</v>
+      </c>
+      <c r="C37" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>4662</v>
+      </c>
+      <c r="F37" t="s" s="0">
+        <v>4663</v>
+      </c>
+      <c r="G37" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>4664</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>4665</v>
+      </c>
+      <c r="C38" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E38" t="s" s="0">
+        <v>4666</v>
+      </c>
+      <c r="F38" t="s" s="0">
+        <v>4667</v>
+      </c>
+      <c r="G38" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>4668</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>4669</v>
+      </c>
+      <c r="C39" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>4666</v>
+      </c>
+      <c r="F39" t="s" s="0">
+        <v>4667</v>
+      </c>
+      <c r="G39" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>4670</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>4671</v>
+      </c>
+      <c r="C40" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D40" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E40" t="s" s="0">
+        <v>4666</v>
+      </c>
+      <c r="F40" t="s" s="0">
+        <v>4667</v>
+      </c>
+      <c r="G40" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>4672</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>4673</v>
+      </c>
+      <c r="C41" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D41" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s" s="0">
+        <v>4674</v>
+      </c>
+      <c r="F41" t="s" s="0">
+        <v>4675</v>
+      </c>
+      <c r="G41" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>4676</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>4677</v>
+      </c>
+      <c r="C42" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E42" t="s" s="0">
+        <v>4678</v>
+      </c>
+      <c r="F42" t="s" s="0">
+        <v>4679</v>
+      </c>
+      <c r="G42" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>4680</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>4681</v>
+      </c>
+      <c r="C43" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D43" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s" s="0">
+        <v>4643</v>
+      </c>
+      <c r="F43" t="s" s="0">
+        <v>4644</v>
+      </c>
+      <c r="G43" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>4682</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>4683</v>
+      </c>
+      <c r="C44" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E44" t="s" s="0">
+        <v>4684</v>
+      </c>
+      <c r="F44" t="s" s="0">
+        <v>4685</v>
+      </c>
+      <c r="G44" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>4686</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>4687</v>
+      </c>
+      <c r="C45" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E45" t="s" s="0">
+        <v>4684</v>
+      </c>
+      <c r="F45" t="s" s="0">
+        <v>4685</v>
+      </c>
+      <c r="G45" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>4688</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>3457</v>
+      </c>
+      <c r="C46" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s" s="0">
+        <v>4689</v>
+      </c>
+      <c r="F46" t="s" s="0">
+        <v>4690</v>
+      </c>
+      <c r="G46" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>4691</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>4692</v>
+      </c>
+      <c r="C47" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s" s="0">
+        <v>4689</v>
+      </c>
+      <c r="F47" t="s" s="0">
+        <v>4690</v>
+      </c>
+      <c r="G47" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>4693</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>4694</v>
+      </c>
+      <c r="C48" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E48" t="s" s="0">
+        <v>4689</v>
+      </c>
+      <c r="F48" t="s" s="0">
+        <v>4690</v>
+      </c>
+      <c r="G48" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>4695</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>4696</v>
+      </c>
+      <c r="C49" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s" s="0">
+        <v>4697</v>
+      </c>
+      <c r="F49" t="s" s="0">
+        <v>4698</v>
+      </c>
+      <c r="G49" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>4699</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>4700</v>
+      </c>
+      <c r="C50" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s" s="0">
+        <v>4697</v>
+      </c>
+      <c r="F50" t="s" s="0">
+        <v>4698</v>
+      </c>
+      <c r="G50" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>4701</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>4702</v>
+      </c>
+      <c r="C51" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s" s="0">
+        <v>4703</v>
+      </c>
+      <c r="F51" t="s" s="0">
+        <v>4704</v>
+      </c>
+      <c r="G51" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>4705</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>4706</v>
+      </c>
+      <c r="C52" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s" s="0">
+        <v>4707</v>
+      </c>
+      <c r="F52" t="s" s="0">
+        <v>4708</v>
+      </c>
+      <c r="G52" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>4709</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>4710</v>
+      </c>
+      <c r="C53" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s" s="0">
+        <v>4707</v>
+      </c>
+      <c r="F53" t="s" s="0">
+        <v>4708</v>
+      </c>
+      <c r="G53" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>4711</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>4712</v>
+      </c>
+      <c r="C54" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E54" t="s" s="0">
+        <v>4713</v>
+      </c>
+      <c r="F54" t="s" s="0">
+        <v>4714</v>
+      </c>
+      <c r="G54" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>4715</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>4716</v>
+      </c>
+      <c r="C55" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s" s="0">
+        <v>4717</v>
+      </c>
+      <c r="F55" t="s" s="0">
+        <v>4718</v>
+      </c>
+      <c r="G55" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>4719</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>4720</v>
+      </c>
+      <c r="C56" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E56" t="s" s="0">
+        <v>4721</v>
+      </c>
+      <c r="F56" t="s" s="0">
+        <v>4722</v>
+      </c>
+      <c r="G56" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>4723</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>4724</v>
+      </c>
+      <c r="C57" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D57" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s" s="0">
+        <v>4721</v>
+      </c>
+      <c r="F57" t="s" s="0">
+        <v>4722</v>
+      </c>
+      <c r="G57" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>4725</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>4726</v>
+      </c>
+      <c r="C58" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D58" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E58" t="s" s="0">
+        <v>4721</v>
+      </c>
+      <c r="F58" t="s" s="0">
+        <v>4722</v>
+      </c>
+      <c r="G58" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>4727</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>4728</v>
+      </c>
+      <c r="C59" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E59" t="s" s="0">
+        <v>4729</v>
+      </c>
+      <c r="F59" t="s" s="0">
+        <v>4730</v>
+      </c>
+      <c r="G59" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>4731</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>4732</v>
+      </c>
+      <c r="C60" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E60" t="s" s="0">
+        <v>4733</v>
+      </c>
+      <c r="F60" t="s" s="0">
+        <v>4734</v>
+      </c>
+      <c r="G60" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="0">
+        <v>4735</v>
+      </c>
+      <c r="B61" t="s" s="0">
+        <v>4736</v>
+      </c>
+      <c r="C61" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E61" t="s" s="0">
+        <v>4737</v>
+      </c>
+      <c r="F61" t="s" s="0">
+        <v>4738</v>
+      </c>
+      <c r="G61" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="0">
+        <v>4739</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>4740</v>
+      </c>
+      <c r="C62" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E62" t="s" s="0">
+        <v>4733</v>
+      </c>
+      <c r="F62" t="s" s="0">
+        <v>4734</v>
+      </c>
+      <c r="G62" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>4741</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>4742</v>
+      </c>
+      <c r="C63" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D63" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E63" t="s" s="0">
+        <v>4743</v>
+      </c>
+      <c r="F63" t="s" s="0">
+        <v>4744</v>
+      </c>
+      <c r="G63" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>4745</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>4746</v>
+      </c>
+      <c r="C64" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="D64" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E64" t="s" s="0">
+        <v>4743</v>
+      </c>
+      <c r="F64" t="s" s="0">
+        <v>4744</v>
+      </c>
+      <c r="G64" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F32FDA50-4CE5-4C6A-9341-BE89D4EFCBE3}">
   <dimension ref="A1:G26"/>

</xml_diff>